<commit_message>
new data,new graph and a bit of the text
</commit_message>
<xml_diff>
--- a/Taxi Data.xlsx
+++ b/Taxi Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d53e1b5d2246abec/Documents/Personal/projects of sorts/uber-pricing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="8_{3B24423F-813C-4F1A-B4CB-FEFE64AFEF18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A836B7ED-6931-4E5A-AC63-9C843ADBACFE}"/>
+  <xr:revisionPtr revIDLastSave="200" documentId="8_{3B24423F-813C-4F1A-B4CB-FEFE64AFEF18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8C04A6F-643C-4775-815F-0C36CFA2662D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{470FE2EC-4CBC-4582-9FEB-C929F3C24366}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="21">
   <si>
     <t>miles</t>
   </si>
@@ -93,6 +93,15 @@
   </si>
   <si>
     <t>portugal</t>
+  </si>
+  <si>
+    <t>england</t>
+  </si>
+  <si>
+    <t>Hamish</t>
+  </si>
+  <si>
+    <t>Harrison</t>
   </si>
 </sst>
 </file>
@@ -143,13 +152,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -165,6 +173,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -484,7 +496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0F1307C-E83B-4FBC-B3F6-4FA02731CB36}">
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.77734375" bestFit="1" customWidth="1"/>
@@ -948,7 +960,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>26.58</v>
       </c>
@@ -978,7 +990,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B18" s="4">
         <v>11.9</v>
       </c>
@@ -1004,7 +1016,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B19" s="4">
         <v>10.9</v>
       </c>
@@ -1030,7 +1042,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B20" s="4">
         <v>8.9600000000000009</v>
       </c>
@@ -1056,7 +1068,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B21" s="4">
         <v>7.98</v>
       </c>
@@ -1082,7 +1094,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B22" s="4">
         <v>5.92</v>
       </c>
@@ -1108,7 +1120,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B23" s="4">
         <v>5.44</v>
       </c>
@@ -1124,7 +1136,7 @@
       <c r="F23" s="3">
         <v>45963</v>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="2">
         <v>7.0833333333333331E-2</v>
       </c>
       <c r="H23" t="s">
@@ -1134,7 +1146,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>4.99</v>
       </c>
@@ -1162,11 +1174,8 @@
       <c r="I24" t="s">
         <v>15</v>
       </c>
-      <c r="J24">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>4.07</v>
       </c>
@@ -1195,11 +1204,8 @@
       <c r="I25" t="s">
         <v>15</v>
       </c>
-      <c r="J25">
-        <v>3.09</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B26" s="4">
         <v>5.96</v>
       </c>
@@ -1225,8 +1231,502 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="G27" s="2"/>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B27" s="4">
+        <v>24.95</v>
+      </c>
+      <c r="C27">
+        <v>11.11</v>
+      </c>
+      <c r="D27">
+        <v>19</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F27" s="3">
+        <v>46253</v>
+      </c>
+      <c r="G27" s="2">
+        <v>0.46111111111111114</v>
+      </c>
+      <c r="H27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I27" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B28" s="4">
+        <v>7.94</v>
+      </c>
+      <c r="C28">
+        <v>2.02</v>
+      </c>
+      <c r="D28">
+        <v>8</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F28" s="3">
+        <v>46239</v>
+      </c>
+      <c r="G28" s="2">
+        <v>0.61944444444444446</v>
+      </c>
+      <c r="H28" t="s">
+        <v>19</v>
+      </c>
+      <c r="I28" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B29" s="4">
+        <v>41.99</v>
+      </c>
+      <c r="C29">
+        <v>12.57</v>
+      </c>
+      <c r="D29">
+        <v>24</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F29" s="3">
+        <v>46222</v>
+      </c>
+      <c r="G29" s="2">
+        <v>1.3888888888888889E-3</v>
+      </c>
+      <c r="H29" t="s">
+        <v>19</v>
+      </c>
+      <c r="I29" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B30" s="4">
+        <v>34.35</v>
+      </c>
+      <c r="C30">
+        <v>12.42</v>
+      </c>
+      <c r="D30">
+        <v>24</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" s="3">
+        <v>46221</v>
+      </c>
+      <c r="G30" s="2">
+        <v>0.82916666666666672</v>
+      </c>
+      <c r="H30" t="s">
+        <v>19</v>
+      </c>
+      <c r="I30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B31" s="4">
+        <v>5.54</v>
+      </c>
+      <c r="C31">
+        <v>1.29</v>
+      </c>
+      <c r="D31">
+        <v>5</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F31" s="3">
+        <v>46197</v>
+      </c>
+      <c r="G31" s="2">
+        <v>0.35972222222222222</v>
+      </c>
+      <c r="H31" t="s">
+        <v>19</v>
+      </c>
+      <c r="I31" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B32" s="4">
+        <v>27.41</v>
+      </c>
+      <c r="C32">
+        <v>21.5</v>
+      </c>
+      <c r="D32">
+        <v>36</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F32" s="3">
+        <v>46202</v>
+      </c>
+      <c r="G32" s="2">
+        <v>0.47499999999999998</v>
+      </c>
+      <c r="H32" t="s">
+        <v>19</v>
+      </c>
+      <c r="I32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B33" s="4">
+        <v>26.07</v>
+      </c>
+      <c r="C33">
+        <v>13.97</v>
+      </c>
+      <c r="D33">
+        <v>24</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F33" s="3">
+        <v>46187</v>
+      </c>
+      <c r="G33" s="2">
+        <v>0.30208333333333331</v>
+      </c>
+      <c r="H33" t="s">
+        <v>19</v>
+      </c>
+      <c r="I33" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B34" s="4">
+        <v>22.9</v>
+      </c>
+      <c r="C34">
+        <v>18.329999999999998</v>
+      </c>
+      <c r="D34">
+        <v>34</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F34" s="3">
+        <v>46180</v>
+      </c>
+      <c r="G34" s="2">
+        <v>0.30555555555555558</v>
+      </c>
+      <c r="H34" t="s">
+        <v>19</v>
+      </c>
+      <c r="I34" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B35" s="4">
+        <v>40.950000000000003</v>
+      </c>
+      <c r="C35">
+        <v>22.13</v>
+      </c>
+      <c r="D35">
+        <v>32</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F35" s="3">
+        <v>46164</v>
+      </c>
+      <c r="G35" s="2">
+        <v>0.82708333333333328</v>
+      </c>
+      <c r="H35" t="s">
+        <v>19</v>
+      </c>
+      <c r="I35" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B36" s="4">
+        <v>5.93</v>
+      </c>
+      <c r="C36">
+        <v>1.27</v>
+      </c>
+      <c r="D36">
+        <v>5</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F36" s="3">
+        <v>46149</v>
+      </c>
+      <c r="G36" s="2">
+        <v>0.3125</v>
+      </c>
+      <c r="H36" t="s">
+        <v>19</v>
+      </c>
+      <c r="I36" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B37" s="4">
+        <v>15.43</v>
+      </c>
+      <c r="C37">
+        <v>1.52</v>
+      </c>
+      <c r="D37">
+        <v>4</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F37" s="3">
+        <v>46146</v>
+      </c>
+      <c r="G37" s="2">
+        <v>0.28125</v>
+      </c>
+      <c r="H37" t="s">
+        <v>19</v>
+      </c>
+      <c r="I37" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B38" s="4">
+        <v>16.79</v>
+      </c>
+      <c r="C38">
+        <v>7.14</v>
+      </c>
+      <c r="D38">
+        <v>21</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F38" s="3">
+        <v>46080</v>
+      </c>
+      <c r="G38" s="2">
+        <v>0.46041666666666664</v>
+      </c>
+      <c r="H38" t="s">
+        <v>19</v>
+      </c>
+      <c r="I38" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B39" s="4">
+        <v>5.94</v>
+      </c>
+      <c r="C39">
+        <v>1.28</v>
+      </c>
+      <c r="D39">
+        <v>4</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F39" s="3">
+        <v>46069</v>
+      </c>
+      <c r="G39" s="2">
+        <v>0.82708333333333328</v>
+      </c>
+      <c r="H39" t="s">
+        <v>19</v>
+      </c>
+      <c r="I39" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B40" s="4">
+        <v>6.11</v>
+      </c>
+      <c r="C40">
+        <v>1.28</v>
+      </c>
+      <c r="D40">
+        <v>4</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F40" s="3">
+        <v>46055</v>
+      </c>
+      <c r="G40" s="2">
+        <v>0.82499999999999996</v>
+      </c>
+      <c r="H40" t="s">
+        <v>19</v>
+      </c>
+      <c r="I40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B41" s="4">
+        <v>4.95</v>
+      </c>
+      <c r="C41">
+        <v>1.29</v>
+      </c>
+      <c r="D41">
+        <v>4</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F41" s="3">
+        <v>46050</v>
+      </c>
+      <c r="G41" s="2">
+        <v>0.28819444444444442</v>
+      </c>
+      <c r="H41" t="s">
+        <v>19</v>
+      </c>
+      <c r="I41" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B42" s="4">
+        <v>15.95</v>
+      </c>
+      <c r="C42">
+        <v>7.52</v>
+      </c>
+      <c r="D42">
+        <v>20</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F42" s="3">
+        <v>46049</v>
+      </c>
+      <c r="G42" s="2">
+        <v>0.62916666666666665</v>
+      </c>
+      <c r="H42" t="s">
+        <v>19</v>
+      </c>
+      <c r="I42" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B43" s="4">
+        <v>4.9800000000000004</v>
+      </c>
+      <c r="C43">
+        <v>1.35</v>
+      </c>
+      <c r="D43">
+        <v>4</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F43" s="3">
+        <v>46044</v>
+      </c>
+      <c r="G43" s="2">
+        <v>0.82847222222222228</v>
+      </c>
+      <c r="H43" t="s">
+        <v>19</v>
+      </c>
+      <c r="I43" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B44" s="4">
+        <v>3.57</v>
+      </c>
+      <c r="C44">
+        <v>2.17</v>
+      </c>
+      <c r="D44">
+        <v>8</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F44" s="3">
+        <v>46180</v>
+      </c>
+      <c r="G44" s="2">
+        <v>0.45763888888888887</v>
+      </c>
+      <c r="H44" t="s">
+        <v>20</v>
+      </c>
+      <c r="I44" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>3.4</v>
+      </c>
+      <c r="B45" s="4">
+        <v>2.94</v>
+      </c>
+      <c r="C45">
+        <v>2.5</v>
+      </c>
+      <c r="D45">
+        <v>7</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F45" s="3">
+        <v>46178</v>
+      </c>
+      <c r="G45" s="2">
+        <v>0.46944444444444444</v>
+      </c>
+      <c r="H45" t="s">
+        <v>20</v>
+      </c>
+      <c r="I45" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>